<commit_message>
Update outputs with corrected xlsx timestamps
</commit_message>
<xml_diff>
--- a/outputs/20260817/data_extent_summary.xlsx
+++ b/outputs/20260817/data_extent_summary.xlsx
@@ -400,10 +400,10 @@
         <v>7091666</v>
       </c>
       <c r="C2" s="2">
-        <v>45717.07297445602</v>
+        <v>45717.28129629629</v>
       </c>
       <c r="D2" s="2">
-        <v>46249.63787868056</v>
+        <v>46249.8462037037</v>
       </c>
       <c r="E2">
         <v>532.6</v>
@@ -419,10 +419,10 @@
         <v>269473</v>
       </c>
       <c r="C3" s="2">
-        <v>45931.06275387731</v>
+        <v>45931.27107638889</v>
       </c>
       <c r="D3" s="2">
-        <v>46234.62998724537</v>
+        <v>46234.83831018519</v>
       </c>
       <c r="E3">
         <v>303.6</v>
@@ -438,10 +438,10 @@
         <v>7736270</v>
       </c>
       <c r="C4" s="2">
-        <v>45930.79176180555</v>
+        <v>45931.00009259259</v>
       </c>
       <c r="D4" s="2">
-        <v>46234.79163703704</v>
+        <v>46234.99996527778</v>
       </c>
       <c r="E4">
         <v>304</v>
@@ -454,16 +454,16 @@
         </is>
       </c>
       <c r="B5">
-        <v>115130</v>
+        <v>213766</v>
       </c>
       <c r="C5" s="2">
-        <v>45930.79167824074</v>
+        <v>45658</v>
       </c>
       <c r="D5" s="2">
-        <v>46249.77085648148</v>
+        <v>46249.97918981481</v>
       </c>
       <c r="E5">
-        <v>319</v>
+        <v>592</v>
       </c>
     </row>
   </sheetData>
@@ -517,10 +517,10 @@
         <v>11627</v>
       </c>
       <c r="C2" s="2">
-        <v>45945.07297753472</v>
+        <v>45945.28130787037</v>
       </c>
       <c r="D2" s="2">
-        <v>46234.5770624537</v>
+        <v>46234.78539351852</v>
       </c>
       <c r="E2">
         <v>289.5</v>
@@ -536,10 +536,10 @@
         <v>11627</v>
       </c>
       <c r="C3" s="2">
-        <v>45945.07297753472</v>
+        <v>45945.28130787037</v>
       </c>
       <c r="D3" s="2">
-        <v>46234.5770624537</v>
+        <v>46234.78539351852</v>
       </c>
       <c r="E3">
         <v>289.5</v>
@@ -555,10 +555,10 @@
         <v>6945</v>
       </c>
       <c r="C4" s="2">
-        <v>45945.20787368056</v>
+        <v>45945.4162037037</v>
       </c>
       <c r="D4" s="2">
-        <v>46232.15430511574</v>
+        <v>46232.36262731481</v>
       </c>
       <c r="E4">
         <v>286.9</v>
@@ -574,10 +574,10 @@
         <v>2315</v>
       </c>
       <c r="C5" s="2">
-        <v>45945.20787368056</v>
+        <v>45945.4162037037</v>
       </c>
       <c r="D5" s="2">
-        <v>46232.15430511574</v>
+        <v>46232.36262731481</v>
       </c>
       <c r="E5">
         <v>286.9</v>
@@ -593,10 +593,10 @@
         <v>3487</v>
       </c>
       <c r="C6" s="2">
-        <v>45953.26626944444</v>
+        <v>45953.47459490741</v>
       </c>
       <c r="D6" s="2">
-        <v>46237.58823267361</v>
+        <v>46237.7965625</v>
       </c>
       <c r="E6">
         <v>284.3</v>

</xml_diff>